<commit_message>
fix(audit-v6): resolve cross-lineage reporting, caliper horizon, concordance metrics, intra-array statistics, verifier robustness, and PDF formatting
</commit_message>
<xml_diff>
--- a/data/Supplementary_Tables_S1_to_S8.xlsx
+++ b/data/Supplementary_Tables_S1_to_S8.xlsx
@@ -2448,14 +2448,14 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>74696</v>
+        <v>74763</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>75911</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>98.40%</t>
+          <t>98.49%</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2755,7 +2755,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>57428</v>
+        <v>57426</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>74932</v>

</xml_diff>

<commit_message>
fix(audit-v7): resolve coordinate arithmetic, di-estimator, dynamic concordance, sign-test, html sync, and verifier robustness
</commit_message>
<xml_diff>
--- a/data/Supplementary_Tables_S1_to_S8.xlsx
+++ b/data/Supplementary_Tables_S1_to_S8.xlsx
@@ -538,11 +538,15 @@
       <c r="C2" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="D2" s="3" t="n">
-        <v>290</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>160</v>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="F2" s="3" t="n">
         <v>179722</v>
@@ -726,11 +730,15 @@
       <c r="G6" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>310</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>180</v>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -766,11 +774,15 @@
       <c r="G7" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>305</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>175</v>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -1054,11 +1066,15 @@
       <c r="C14" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="D14" s="3" t="n">
-        <v>295</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>165</v>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="F14" s="3" t="n">
         <v>139108</v>
@@ -1330,11 +1346,15 @@
       <c r="G20" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="H20" s="3" t="n">
-        <v>290</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>160</v>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -1530,11 +1550,15 @@
       <c r="C25" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="D25" s="3" t="n">
-        <v>290</v>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>160</v>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
       <c r="F25" s="3" t="n">
         <v>3224999</v>
@@ -1542,14 +1566,20 @@
       <c r="G25" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="H25" s="3" t="n">
-        <v>310</v>
-      </c>
-      <c r="I25" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="J25" s="3" t="n">
-        <v>20</v>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2448,7 +2478,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>74763</v>
+        <v>74765</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>75911</v>
@@ -2758,7 +2788,7 @@
         <v>57426</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>74932</v>
+        <v>74925</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2791,7 +2821,7 @@
         <v>161</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>74932</v>
+        <v>74925</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2821,13 +2851,13 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>11497</v>
+        <v>11456</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>11497</v>
+        <v>11456</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>11497</v>
+        <v>11456</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -2852,13 +2882,13 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>12991</v>
+        <v>12923</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>12991</v>
+        <v>12923</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>12991</v>
+        <v>12923</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -2883,13 +2913,13 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>1347</v>
+        <v>1308</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>1347</v>
+        <v>1308</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>1347</v>
+        <v>1308</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -7896,7 +7926,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -7998,7 +8028,7 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>84780</v>
+        <v>84779</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>133</v>
@@ -8054,7 +8084,7 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>74932</v>
+        <v>74925</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>133</v>
@@ -8074,7 +8104,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>3.02%</t>
+          <t>3.01%</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -8091,7 +8121,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HG002 (GM24385)</t>
+          <t>HG002 (GM24385, EBV-transformed)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -8110,7 +8140,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>11497</v>
+        <v>11456</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>20</v>
@@ -8125,12 +8155,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>0.435%</t>
+          <t>0.436%</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>38.64%</t>
+          <t>38.74%</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -8166,7 +8196,7 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>12991</v>
+        <v>12923</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>175</v>
@@ -8176,17 +8206,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>12.39%</t>
+          <t>12.45%</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>0.608%</t>
+          <t>0.611%</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>7.31%</t>
+          <t>7.11%</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -8222,7 +8252,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1347</v>
+        <v>1308</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>126</v>
@@ -8232,17 +8262,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>12.84%</t>
+          <t>13.23%</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>0.817%</t>
+          <t>0.841%</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2.38%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">

</xml_diff>